<commit_message>
Fix header row handling
</commit_message>
<xml_diff>
--- a/tests/input/HeaderRow.xlsx
+++ b/tests/input/HeaderRow.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/path/to/file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{54AA8755-4CFB-8041-9553-588786C2555F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650D74DF-3818-AB4E-927F-480D05DA0C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1000" yWindow="880" windowWidth="28240" windowHeight="17240" xr2:uid="{6F850C66-F5CE-8944-BF19-5C6406FF5A3E}"/>
+    <workbookView xWindow="1000" yWindow="880" windowWidth="28240" windowHeight="17240" activeTab="2" xr2:uid="{6F850C66-F5CE-8944-BF19-5C6406FF5A3E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="3">
   <si>
     <t>Column A</t>
   </si>
@@ -565,4 +566,71 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8F714A4-03ED-7646-BB55-296B80D35A70}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B2">
+        <v>-42</v>
+      </c>
+      <c r="C2">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>30</v>
+      </c>
+      <c r="B4">
+        <v>9.8378440000000005</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>-273.14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>50</v>
+      </c>
+      <c r="B6">
+        <v>99.99</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>